<commit_message>
Pre-fill Template 7 prerequisites from 2026-27 course catalog
Extracted 67 prerequisite entries and 3 corequisite entries from the
Don Bosco Prep 2026-2027 Course Catalog PDF into Template 7 (Course
Profiles) columns 20-21. Covers all departments: Business, Comm Arts,
Computer Science, Engineering, Math, Music/Art, Science, Social Studies,
Theater, and World Languages.

Also changed v3 engine credit cap validation from hard halt to warning,
since 82% of students request more courses than 7 periods allow (normal
wish-list behavior). Cap remains at 35.0 credits per user confirmation.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_7_Course_Profiles.xlsx
+++ b/templates/Template_7_Course_Profiles.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -147,6 +147,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3107,9 +3110,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T22" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T22" s="8" t="inlineStr">
+        <is>
+          <t>201</t>
         </is>
       </c>
       <c r="U22" s="7" t="inlineStr">
@@ -3687,9 +3690,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T27" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T27" s="8" t="inlineStr">
+        <is>
+          <t>225</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
@@ -3919,9 +3922,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T29" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T29" s="8" t="inlineStr">
+        <is>
+          <t>241</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
@@ -4035,9 +4038,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T30" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T30" s="8" t="inlineStr">
+        <is>
+          <t>242</t>
         </is>
       </c>
       <c r="U30" s="7" t="inlineStr">
@@ -4151,9 +4154,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T31" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T31" s="8" t="inlineStr">
+        <is>
+          <t>241</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
@@ -4267,9 +4270,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T32" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T32" s="8" t="inlineStr">
+        <is>
+          <t>241</t>
         </is>
       </c>
       <c r="U32" s="7" t="inlineStr">
@@ -4383,9 +4386,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T33" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T33" s="8" t="inlineStr">
+        <is>
+          <t>242,243</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
@@ -4499,9 +4502,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T34" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T34" s="8" t="inlineStr">
+        <is>
+          <t>242,243</t>
         </is>
       </c>
       <c r="U34" s="7" t="inlineStr">
@@ -4615,9 +4618,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T35" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T35" s="8" t="inlineStr">
+        <is>
+          <t>242,243</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
@@ -5195,9 +5198,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T40" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T40" s="8" t="inlineStr">
+        <is>
+          <t>310,311</t>
         </is>
       </c>
       <c r="U40" s="7" t="inlineStr">
@@ -5311,9 +5314,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T41" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T41" s="8" t="inlineStr">
+        <is>
+          <t>310,311</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
@@ -5427,9 +5430,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T42" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T42" s="8" t="inlineStr">
+        <is>
+          <t>312</t>
         </is>
       </c>
       <c r="U42" s="7" t="inlineStr">
@@ -5543,9 +5546,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T43" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T43" s="8" t="inlineStr">
+        <is>
+          <t>312</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
@@ -5659,9 +5662,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T44" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T44" s="8" t="inlineStr">
+        <is>
+          <t>315</t>
         </is>
       </c>
       <c r="U44" s="7" t="inlineStr">
@@ -5775,9 +5778,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T45" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T45" s="8" t="inlineStr">
+        <is>
+          <t>320,321</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
@@ -5891,9 +5894,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T46" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T46" s="8" t="inlineStr">
+        <is>
+          <t>320,321</t>
         </is>
       </c>
       <c r="U46" s="7" t="inlineStr">
@@ -6007,9 +6010,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T47" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T47" s="8" t="inlineStr">
+        <is>
+          <t>322,323</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
@@ -6123,9 +6126,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T48" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T48" s="8" t="inlineStr">
+        <is>
+          <t>322,323</t>
         </is>
       </c>
       <c r="U48" s="7" t="inlineStr">
@@ -6239,9 +6242,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T49" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T49" s="8" t="inlineStr">
+        <is>
+          <t>327</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
@@ -6355,9 +6358,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T50" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T50" s="8" t="inlineStr">
+        <is>
+          <t>331</t>
         </is>
       </c>
       <c r="U50" s="7" t="inlineStr">
@@ -6471,9 +6474,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T51" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T51" s="8" t="inlineStr">
+        <is>
+          <t>333</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
@@ -6587,9 +6590,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T52" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T52" s="8" t="inlineStr">
+        <is>
+          <t>339</t>
         </is>
       </c>
       <c r="U52" s="7" t="inlineStr">
@@ -7051,9 +7054,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T56" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T56" s="8" t="inlineStr">
+        <is>
+          <t>410,411,412</t>
         </is>
       </c>
       <c r="U56" s="7" t="inlineStr">
@@ -7167,9 +7170,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T57" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T57" s="8" t="inlineStr">
+        <is>
+          <t>411</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
@@ -7399,9 +7402,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T59" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T59" s="8" t="inlineStr">
+        <is>
+          <t>410,411</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
@@ -7515,9 +7518,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T60" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T60" s="8" t="inlineStr">
+        <is>
+          <t>420,421,422,425</t>
         </is>
       </c>
       <c r="U60" s="7" t="inlineStr">
@@ -7631,9 +7634,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T61" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T61" s="8" t="inlineStr">
+        <is>
+          <t>421,425</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
@@ -7747,9 +7750,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T62" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T62" s="8" t="inlineStr">
+        <is>
+          <t>420,421,422,425</t>
         </is>
       </c>
       <c r="U62" s="7" t="inlineStr">
@@ -7863,9 +7866,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T63" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T63" s="8" t="inlineStr">
+        <is>
+          <t>425,421</t>
         </is>
       </c>
       <c r="U63" s="7" t="inlineStr">
@@ -7979,9 +7982,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T64" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T64" s="8" t="inlineStr">
+        <is>
+          <t>430,431,432,435</t>
         </is>
       </c>
       <c r="U64" s="7" t="inlineStr">
@@ -8095,9 +8098,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T65" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T65" s="8" t="inlineStr">
+        <is>
+          <t>430,431,432,435</t>
         </is>
       </c>
       <c r="U65" s="7" t="inlineStr">
@@ -8211,9 +8214,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T66" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T66" s="8" t="inlineStr">
+        <is>
+          <t>435</t>
         </is>
       </c>
       <c r="U66" s="7" t="inlineStr">
@@ -8443,9 +8446,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T68" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T68" s="8" t="inlineStr">
+        <is>
+          <t>440,443,445</t>
         </is>
       </c>
       <c r="U68" s="7" t="inlineStr">
@@ -8559,9 +8562,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T69" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T69" s="8" t="inlineStr">
+        <is>
+          <t>445</t>
         </is>
       </c>
       <c r="U69" s="7" t="inlineStr">
@@ -8675,9 +8678,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T70" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T70" s="8" t="inlineStr">
+        <is>
+          <t>445</t>
         </is>
       </c>
       <c r="U70" s="7" t="inlineStr">
@@ -8791,9 +8794,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T71" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T71" s="8" t="inlineStr">
+        <is>
+          <t>453,455</t>
         </is>
       </c>
       <c r="U71" s="7" t="inlineStr">
@@ -9139,9 +9142,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T74" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T74" s="8" t="inlineStr">
+        <is>
+          <t>473,580</t>
         </is>
       </c>
       <c r="U74" s="7" t="inlineStr">
@@ -9255,9 +9258,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T75" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T75" s="8" t="inlineStr">
+        <is>
+          <t>473,580</t>
         </is>
       </c>
       <c r="U75" s="7" t="inlineStr">
@@ -9371,9 +9374,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T76" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T76" s="8" t="inlineStr">
+        <is>
+          <t>472,473,580</t>
         </is>
       </c>
       <c r="U76" s="7" t="inlineStr">
@@ -9487,9 +9490,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T77" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T77" s="8" t="inlineStr">
+        <is>
+          <t>490,491,580</t>
         </is>
       </c>
       <c r="U77" s="7" t="inlineStr">
@@ -10067,9 +10070,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T82" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T82" s="8" t="inlineStr">
+        <is>
+          <t>511</t>
         </is>
       </c>
       <c r="U82" s="7" t="inlineStr">
@@ -10188,9 +10191,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="U83" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="U83" s="8" t="inlineStr">
+        <is>
+          <t>430,431,432,435</t>
         </is>
       </c>
       <c r="V83" s="7" t="inlineStr">
@@ -10304,9 +10307,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="U84" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="U84" s="8" t="inlineStr">
+        <is>
+          <t>430,431,432,435</t>
         </is>
       </c>
       <c r="V84" s="7" t="inlineStr">
@@ -10415,9 +10418,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T85" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T85" s="8" t="inlineStr">
+        <is>
+          <t>510,511,520,521</t>
         </is>
       </c>
       <c r="U85" s="7" t="inlineStr">
@@ -10531,9 +10534,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T86" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T86" s="8" t="inlineStr">
+        <is>
+          <t>510,511,520,521</t>
         </is>
       </c>
       <c r="U86" s="7" t="inlineStr">
@@ -10879,9 +10882,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T89" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T89" s="8" t="inlineStr">
+        <is>
+          <t>511</t>
         </is>
       </c>
       <c r="U89" s="7" t="inlineStr">
@@ -10995,9 +10998,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T90" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T90" s="8" t="inlineStr">
+        <is>
+          <t>521</t>
         </is>
       </c>
       <c r="U90" s="7" t="inlineStr">
@@ -11111,9 +11114,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T91" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T91" s="8" t="inlineStr">
+        <is>
+          <t>551,553,521,531,445</t>
         </is>
       </c>
       <c r="U91" s="7" t="inlineStr">
@@ -11227,9 +11230,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T92" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T92" s="8" t="inlineStr">
+        <is>
+          <t>551,553,521,531,445</t>
         </is>
       </c>
       <c r="U92" s="7" t="inlineStr">
@@ -11459,9 +11462,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T94" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T94" s="8" t="inlineStr">
+        <is>
+          <t>410,411,412</t>
         </is>
       </c>
       <c r="U94" s="7" t="inlineStr">
@@ -11575,9 +11578,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T95" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T95" s="8" t="inlineStr">
+        <is>
+          <t>580</t>
         </is>
       </c>
       <c r="U95" s="7" t="inlineStr">
@@ -11691,9 +11694,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T96" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T96" s="8" t="inlineStr">
+        <is>
+          <t>585,490</t>
         </is>
       </c>
       <c r="U96" s="7" t="inlineStr">
@@ -11807,9 +11810,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T97" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T97" s="8" t="inlineStr">
+        <is>
+          <t>590</t>
         </is>
       </c>
       <c r="U97" s="7" t="inlineStr">
@@ -11923,14 +11926,14 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T98" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U98" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T98" s="8" t="inlineStr">
+        <is>
+          <t>530,531</t>
+        </is>
+      </c>
+      <c r="U98" s="8" t="inlineStr">
+        <is>
+          <t>557,558</t>
         </is>
       </c>
       <c r="V98" s="7" t="inlineStr">
@@ -13199,9 +13202,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T109" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T109" s="8" t="inlineStr">
+        <is>
+          <t>710,711,713</t>
         </is>
       </c>
       <c r="U109" s="7" t="inlineStr">
@@ -13547,9 +13550,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T112" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T112" s="8" t="inlineStr">
+        <is>
+          <t>708</t>
         </is>
       </c>
       <c r="U112" s="7" t="inlineStr">
@@ -14011,9 +14014,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T116" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T116" s="8" t="inlineStr">
+        <is>
+          <t>722,721</t>
         </is>
       </c>
       <c r="U116" s="7" t="inlineStr">
@@ -14127,9 +14130,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T117" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T117" s="8" t="inlineStr">
+        <is>
+          <t>708</t>
         </is>
       </c>
       <c r="U117" s="7" t="inlineStr">
@@ -14475,9 +14478,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T120" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T120" s="8" t="inlineStr">
+        <is>
+          <t>731</t>
         </is>
       </c>
       <c r="U120" s="7" t="inlineStr">
@@ -14707,9 +14710,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T122" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T122" s="8" t="inlineStr">
+        <is>
+          <t>734</t>
         </is>
       </c>
       <c r="U122" s="7" t="inlineStr">
@@ -15171,9 +15174,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T126" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T126" s="8" t="inlineStr">
+        <is>
+          <t>729</t>
         </is>
       </c>
       <c r="U126" s="7" t="inlineStr">
@@ -15403,9 +15406,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T128" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T128" s="8" t="inlineStr">
+        <is>
+          <t>131,139</t>
         </is>
       </c>
       <c r="U128" s="7" t="inlineStr">
@@ -15519,9 +15522,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T129" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T129" s="8" t="inlineStr">
+        <is>
+          <t>733,731</t>
         </is>
       </c>
       <c r="U129" s="7" t="inlineStr">
@@ -15635,9 +15638,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T130" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T130" s="8" t="inlineStr">
+        <is>
+          <t>713,722,733,711,721,731</t>
         </is>
       </c>
       <c r="U130" s="7" t="inlineStr">
@@ -15751,9 +15754,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T131" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T131" s="8" t="inlineStr">
+        <is>
+          <t>733,731</t>
         </is>
       </c>
       <c r="U131" s="7" t="inlineStr">
@@ -15867,9 +15870,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T132" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T132" s="8" t="inlineStr">
+        <is>
+          <t>733,731</t>
         </is>
       </c>
       <c r="U132" s="7" t="inlineStr">
@@ -16795,9 +16798,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T140" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T140" s="8" t="inlineStr">
+        <is>
+          <t>2014</t>
         </is>
       </c>
       <c r="U140" s="7" t="inlineStr">
@@ -16911,9 +16914,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T141" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T141" s="8" t="inlineStr">
+        <is>
+          <t>2024</t>
         </is>
       </c>
       <c r="U141" s="7" t="inlineStr">
@@ -17027,9 +17030,9 @@
           <t>AI CHOICE</t>
         </is>
       </c>
-      <c r="T142" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="T142" s="8" t="inlineStr">
+        <is>
+          <t>2034</t>
         </is>
       </c>
       <c r="U142" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Fix Chiaravalloti section counts: 631 (4 sections) + 642 (6 sections)
- Template 6 Sheet 2: Added 5 rows — 2 more 631 + 3 more 642
  (was 2+3=5, now 4+6=10 semester sections)
- Template 7: Sections Needed 631: 3→4, 642: 3→6
- priority_assignments.json: Updated section counts to match
- semester_designations.json: Updated splits (631: 2×S1+2×S2,
  642: 3×S1+3×S2) for 5 periods per semester
- CLAUDE.md: Documented teacher section prescription

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_7_Course_Profiles.xlsx
+++ b/templates/Template_7_Course_Profiles.xlsx
@@ -6701,7 +6701,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H109" t="n">
         <v>25</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H110" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
Remove 556 AP Physics from Template 7 — AP Physics is only 557
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_7_Course_Profiles.xlsx
+++ b/templates/Template_7_Course_Profiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O147"/>
+  <dimension ref="A1:O146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6043,12 +6043,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>557</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>AP Physics</t>
+          <t>AP Physics 1</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G98" t="n">
@@ -6095,16 +6095,21 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>558</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>AP Physics 1</t>
+          <t>AP Physics C</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6122,18 +6127,18 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H99" t="n">
         <v>25</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -6160,73 +6165,63 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>570</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>AP Physics C</t>
+          <t>Introduction to Robotics</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10,9</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H100" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>Science</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
           <t>Y</t>
-        </is>
-      </c>
-      <c r="N100" t="inlineStr">
-        <is>
-          <t>531</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>580</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Introduction to Robotics</t>
+          <t>Robotics Engineering</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6244,11 +6239,11 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>10,9</t>
+          <t>10,11,9</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H101" t="n">
         <v>20</v>
@@ -6268,16 +6263,21 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>410</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>585</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Robotics Engineering</t>
+          <t>Robotics Design</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -6295,11 +6295,11 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>10,11,9</t>
+          <t>10,11,12</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H102" t="n">
         <v>20</v>
@@ -6321,19 +6321,19 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>580</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>585</t>
+          <t>590</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Robotics Design</t>
+          <t>Robotics Project</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>10,11,12</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G103" t="n">
@@ -6370,6 +6370,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Robotics Block</t>
+        </is>
+      </c>
       <c r="M103" t="inlineStr">
         <is>
           <t>Y</t>
@@ -6377,19 +6382,19 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>585</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>591</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Robotics Project</t>
+          <t>Robotics Project II</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6407,7 +6412,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G104" t="n">
@@ -6438,19 +6443,19 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>585</t>
+          <t>590</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>591</t>
+          <t>595</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Robotics Project II</t>
+          <t>Engineering Design</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6487,36 +6492,31 @@
           <t>N</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>Robotics Block</t>
-        </is>
-      </c>
       <c r="M105" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>590</t>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>530</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>610</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Engineering Design</t>
+          <t>Health/PE</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -6529,14 +6529,14 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H106" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -6548,26 +6548,26 @@
           <t>N</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="O106" t="inlineStr">
-        <is>
-          <t>530</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>620</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Health/PE</t>
+          <t>Driver's Ed/PE</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -6585,11 +6585,11 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H107" t="n">
         <v>25</v>
@@ -6618,12 +6618,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>620</t>
+          <t>631</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Driver's Ed/PE</t>
+          <t>CPR-AED Training/PE</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -6641,11 +6641,11 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H108" t="n">
         <v>25</v>
@@ -6674,12 +6674,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>631</t>
+          <t>642</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>CPR-AED Training/PE</t>
+          <t>Nutrition &amp; Fitness/PE</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -6697,11 +6697,11 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H109" t="n">
         <v>25</v>
@@ -6730,17 +6730,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>708</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Nutrition &amp; Fitness/PE</t>
+          <t>Introduction to Business</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -6753,11 +6753,11 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10,11,12,9</t>
         </is>
       </c>
       <c r="G110" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H110" t="n">
         <v>25</v>
@@ -6772,48 +6772,43 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
-        </is>
-      </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>708</t>
+          <t>710</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Introduction to Business</t>
+          <t>World History</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>10,11,12,9</t>
+          <t>10,9</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H111" t="n">
         <v>25</v>
@@ -6826,6 +6821,11 @@
       <c r="J111" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
@@ -6837,12 +6837,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>711</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>World History</t>
+          <t>World History H</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -6864,7 +6864,7 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H112" t="n">
         <v>25</v>
@@ -6893,12 +6893,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>711</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>World History H</t>
+          <t>AP World History</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6932,7 +6932,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -6949,12 +6949,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>720</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>AP World History</t>
+          <t>U.S. History I</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6972,11 +6972,11 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>10,9</t>
+          <t>10,11</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H114" t="n">
         <v>25</v>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7005,12 +7005,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>U.S. History I</t>
+          <t>U.S. History I H</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7032,7 +7032,7 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H115" t="n">
         <v>25</v>
@@ -7061,12 +7061,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>722</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>U.S. History I H</t>
+          <t>Adv U.S. History I H</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7084,11 +7084,11 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>10,11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H116" t="n">
         <v>25</v>
@@ -7117,12 +7117,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>723</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Adv U.S. History I H</t>
+          <t>Introduction to Political Science</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -7131,20 +7131,20 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10,11,12</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H117" t="n">
         <v>25</v>
@@ -7159,31 +7159,26 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
-        </is>
-      </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>723</t>
+          <t>726</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Introduction to Political Science</t>
+          <t>Business Concepts</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -7200,7 +7195,7 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H118" t="n">
         <v>25</v>
@@ -7217,19 +7212,19 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>726</t>
+          <t>727</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Business Concepts</t>
+          <t>Sports and Entertainment Marketing</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -7275,12 +7270,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>729</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sports and Entertainment Marketing</t>
+          <t>AP Business with Personal Finance</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -7289,20 +7284,20 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>10,11,12</t>
+          <t>10,11</t>
         </is>
       </c>
       <c r="G120" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H120" t="n">
         <v>25</v>
@@ -7314,29 +7309,34 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>708</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>729</t>
+          <t>730</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>AP Business with Personal Finance</t>
+          <t>U.S. History II</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -7349,11 +7349,11 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>10,11</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H121" t="n">
         <v>25</v>
@@ -7365,29 +7365,29 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N121" t="inlineStr">
-        <is>
-          <t>708</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>731</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>U.S. History II</t>
+          <t>U.S. History II H</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -7438,25 +7438,25 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>731</t>
+          <t>732</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>U.S. History II H</t>
+          <t>Business Law</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -7480,11 +7480,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
-        </is>
-      </c>
       <c r="M123" t="inlineStr">
         <is>
           <t>Y</t>
@@ -7494,30 +7489,30 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>732</t>
+          <t>733</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Business Law</t>
+          <t>AP U.S. History</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>10,11,12</t>
         </is>
       </c>
       <c r="G124" t="n">
@@ -7533,46 +7528,56 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>722</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>734</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>AP U.S. History</t>
+          <t>Leadership, Entrepreneurship and Opportunity Program I</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>10,11,12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G125" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H125" t="n">
         <v>25</v>
@@ -7584,39 +7589,34 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>728</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>734</t>
+          <t>741</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Leadership, Entrepreneurship and Opportunity Program I</t>
+          <t>Psychology</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -7629,11 +7629,11 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H126" t="n">
         <v>25</v>
@@ -7650,46 +7650,41 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N126" t="inlineStr">
-        <is>
-          <t>728</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>742</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Psychology</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H127" t="n">
         <v>25</v>
@@ -7713,17 +7708,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>742</t>
+          <t>743</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Economics</t>
+          <t>AP European History</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -7740,36 +7735,46 @@
         </is>
       </c>
       <c r="G128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H128" t="n">
         <v>25</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>731</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>744</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>AP European History</t>
+          <t>Sociology</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -7778,64 +7783,54 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10,11,12</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H129" t="n">
         <v>25</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
         <is>
           <t>Y</t>
-        </is>
-      </c>
-      <c r="N129" t="inlineStr">
-        <is>
-          <t>731</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>744</t>
+          <t>745</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Sociology</t>
+          <t>Leadership, Entrepreneurship and Opportunity Program II</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -7848,7 +7843,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>10,11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G130" t="n">
@@ -7867,26 +7862,36 @@
           <t>N</t>
         </is>
       </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>LEO II</t>
+        </is>
+      </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>734</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>745</t>
+          <t>751</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Leadership, Entrepreneurship and Opportunity Program II</t>
+          <t>American Government &amp; Politics</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7899,18 +7904,18 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H131" t="n">
         <v>25</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -7918,70 +7923,60 @@
           <t>N</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>LEO II</t>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N131" t="inlineStr">
-        <is>
-          <t>734</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>752</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>American Government &amp; Politics</t>
+          <t>Economics H</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H132" t="n">
         <v>25</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
           <t>N</t>
-        </is>
-      </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
@@ -7993,25 +7988,25 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>752</t>
+          <t>756</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Economics H</t>
+          <t>Introduction to Law</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -8020,14 +8015,14 @@
         </is>
       </c>
       <c r="G133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H133" t="n">
         <v>25</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -8037,48 +8032,48 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>756</t>
+          <t>757</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Introduction to Law</t>
+          <t>International Business Strategies</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11,12</t>
         </is>
       </c>
       <c r="G134" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H134" t="n">
         <v>25</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -8088,19 +8083,24 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>729</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>757</t>
+          <t>758</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>International Business Strategies</t>
+          <t>Bloomberg Market Concepts</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -8109,20 +8109,20 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>11,12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H135" t="n">
         <v>25</v>
@@ -8139,37 +8139,32 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N135" t="inlineStr">
-        <is>
-          <t>729</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>758</t>
+          <t>761</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Bloomberg Market Concepts</t>
+          <t>AP Psychology</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Social Studies</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -8178,36 +8173,41 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H136" t="n">
         <v>25</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>131</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>761</t>
+          <t>763</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>AP Psychology</t>
+          <t>AP U.S. Government &amp; Politics</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -8229,14 +8229,14 @@
         </is>
       </c>
       <c r="G137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H137" t="n">
         <v>25</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -8244,6 +8244,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Social Studies</t>
+        </is>
+      </c>
       <c r="M137" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8251,19 +8256,19 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>731</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>763</t>
+          <t>764</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>AP U.S. Government &amp; Politics</t>
+          <t>AP Art History</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -8281,18 +8286,18 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H138" t="n">
         <v>25</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -8305,26 +8310,26 @@
           <t>Social Studies</t>
         </is>
       </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>AP Art Block</t>
+        </is>
+      </c>
       <c r="M138" t="inlineStr">
         <is>
           <t>Y</t>
-        </is>
-      </c>
-      <c r="N138" t="inlineStr">
-        <is>
-          <t>731</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>764</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>AP Art History</t>
+          <t>AP Macroeconomics</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -8333,27 +8338,27 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H139" t="n">
         <v>25</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -8361,31 +8366,26 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>Social Studies</t>
-        </is>
-      </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>AP Art Block</t>
-        </is>
-      </c>
       <c r="M139" t="inlineStr">
         <is>
           <t>Y</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>733</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>766</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>AP Macroeconomics</t>
+          <t>AP Microeconomics</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -8436,34 +8436,34 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>810</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>AP Microeconomics</t>
+          <t>Theology 9</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Social Studies</t>
+          <t>Theology</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G141" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H141" t="n">
         <v>25</v>
@@ -8475,29 +8475,29 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Theology</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N141" t="inlineStr">
-        <is>
-          <t>733</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>810</t>
+          <t>820</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Theology 9</t>
+          <t>Theology 10</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G142" t="n">
@@ -8548,12 +8548,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>830</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Theology 10</t>
+          <t>Theology 11</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8571,11 +8571,11 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G143" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H143" t="n">
         <v>25</v>
@@ -8604,12 +8604,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>830</t>
+          <t>849</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Theology 11</t>
+          <t>Catholic Social Teaching</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8618,20 +8618,20 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>FY</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G144" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H144" t="n">
         <v>25</v>
@@ -8660,12 +8660,12 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>849</t>
+          <t>851</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Catholic Social Teaching</t>
+          <t>Spirituality of Vocation</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8716,37 +8716,37 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>851</t>
+          <t>955</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Spirituality of Vocation</t>
+          <t>Academic Support</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Theology</t>
+          <t>Special Education</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>FY</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10,11,12,9</t>
         </is>
       </c>
       <c r="G146" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H146" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
@@ -8758,63 +8758,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>Theology</t>
-        </is>
-      </c>
       <c r="M146" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>955</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Academic Support</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Special Education</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>0</v>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>FY</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>10,11,12,9</t>
-        </is>
-      </c>
-      <c r="G147" t="n">
-        <v>7</v>
-      </c>
-      <c r="H147" t="n">
-        <v>15</v>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M147" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Fix singleton data: remove 17 false singletons, add 723, sync sources
Removed 17 courses with 2-3 sections from singleton list (were getting
+25 points incorrectly): 201, 203, 242, 243, 249, 450, 472, 585, 590,
591, 595, 713, 722, 744, 765, 766, 2014.

Added 723 Introduction to Political Science (1 section, was not flagged).

Synced course_priorities.json and Template 7 so both sources agree on
all 48 singletons (previously 6 were in only one source: 248 JSON-only,
227/411/453/751/2034 T7-only). Also fixed 201 which was still Y in T7.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_7_Course_Profiles.xlsx
+++ b/templates/Template_7_Course_Profiles.xlsx
@@ -1600,7 +1600,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">

</xml_diff>

<commit_message>
Fix stale prescribed terms in Template 7 for 734 and 765
734 LEO I: S1 -> S2 (matches engine SEMESTER_LOCKS)
765 AP Macroeconomics: S1 -> S2 (matches engine SEMESTER_LOCKS)
766 AP Microeconomics already correct at S1.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_7_Course_Profiles.xlsx
+++ b/templates/Template_7_Course_Profiles.xlsx
@@ -7522,7 +7522,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -8296,7 +8296,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">

</xml_diff>